<commit_message>
Add tc_cal_offset column for thermocouple calibration
</commit_message>
<xml_diff>
--- a/sensor_config.xlsx
+++ b/sensor_config.xlsx
@@ -2760,7 +2760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2811,10 +2811,15 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>tc_cal_offset</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>tc_type</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -2860,12 +2865,15 @@
       <c r="I2" t="n">
         <v>200</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Type K for cryogenic LOX</t>
         </is>
@@ -2911,12 +2919,15 @@
       <c r="I3" t="n">
         <v>200</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Type K for LOX ullage</t>
         </is>
@@ -2962,12 +2973,15 @@
       <c r="I4" t="n">
         <v>200</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>LOX injector temp</t>
         </is>
@@ -3013,12 +3027,15 @@
       <c r="I5" t="n">
         <v>2282</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Chamber temperature - high range</t>
         </is>
@@ -3060,12 +3077,15 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Chamber wall temp</t>
         </is>
@@ -3107,12 +3127,15 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Pyrotechnic temp</t>
         </is>
@@ -3154,12 +3177,15 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>LOX ullage temp</t>
         </is>
@@ -3201,12 +3227,15 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>LOX liquid temp (cryo)</t>
         </is>
@@ -3248,12 +3277,15 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr">
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Dragon injector temp</t>
         </is>
@@ -3295,12 +3327,15 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr">
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Ambient reference</t>
         </is>

</xml_diff>

<commit_message>
feat: implement PANDA DAQ UI v2 and add configuration files for load cells, pressure transducers, and sequences
</commit_message>
<xml_diff>
--- a/sensor_config.xlsx
+++ b/sensor_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\ERPL_GC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA88D92-15A8-4D38-BFA0-C865DBBC1444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C0CC751-7630-4237-A0D2-199D27399BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PT_Sensors" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="305">
   <si>
     <t>system</t>
   </si>
@@ -568,9 +568,6 @@
     <t>weight</t>
   </si>
   <si>
-    <t>Fuel tank weight sensor</t>
-  </si>
-  <si>
     <t>LC4</t>
   </si>
   <si>
@@ -932,6 +929,15 @@
   </si>
   <si>
     <t>LOX slow pressurization</t>
+  </si>
+  <si>
+    <t>TLCC</t>
+  </si>
+  <si>
+    <t>tlcc</t>
+  </si>
+  <si>
+    <t>Thrust load cell C</t>
   </si>
 </sst>
 </file>
@@ -1763,7 +1769,7 @@
         <v>4</v>
       </c>
       <c r="J13">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="K13">
         <v>2000</v>
@@ -2475,13 +2481,13 @@
         <v>177</v>
       </c>
       <c r="D4" t="s">
-        <v>178</v>
+        <v>302</v>
       </c>
       <c r="E4" t="s">
-        <v>179</v>
+        <v>303</v>
       </c>
       <c r="F4" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="G4" t="s">
         <v>171</v>
@@ -2499,7 +2505,7 @@
         <v>130</v>
       </c>
       <c r="L4" t="s">
-        <v>181</v>
+        <v>304</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -2510,13 +2516,13 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" t="s">
         <v>182</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>183</v>
-      </c>
-      <c r="E5" t="s">
-        <v>184</v>
       </c>
       <c r="F5" t="s">
         <v>180</v>
@@ -2537,7 +2543,7 @@
         <v>129</v>
       </c>
       <c r="L5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -2548,13 +2554,13 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D6" t="s">
         <v>186</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>187</v>
-      </c>
-      <c r="E6" t="s">
-        <v>188</v>
       </c>
       <c r="F6" t="s">
         <v>152</v>
@@ -2575,7 +2581,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -2586,13 +2592,13 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
+        <v>189</v>
+      </c>
+      <c r="D7" t="s">
         <v>190</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>191</v>
-      </c>
-      <c r="E7" t="s">
-        <v>192</v>
       </c>
       <c r="F7" t="s">
         <v>152</v>
@@ -2613,7 +2619,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
@@ -2627,7 +2633,7 @@
         <v>167</v>
       </c>
       <c r="D8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E8" t="s">
         <v>170</v>
@@ -2651,7 +2657,7 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
@@ -2665,10 +2671,10 @@
         <v>173</v>
       </c>
       <c r="D9" t="s">
+        <v>182</v>
+      </c>
+      <c r="E9" t="s">
         <v>183</v>
-      </c>
-      <c r="E9" t="s">
-        <v>184</v>
       </c>
       <c r="F9" t="s">
         <v>180</v>
@@ -2689,7 +2695,7 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
@@ -2727,7 +2733,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -2738,16 +2744,16 @@
         <v>3</v>
       </c>
       <c r="C11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D11" t="s">
+        <v>197</v>
+      </c>
+      <c r="E11" t="s">
         <v>198</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>199</v>
-      </c>
-      <c r="F11" t="s">
-        <v>200</v>
       </c>
       <c r="G11" t="s">
         <v>171</v>
@@ -2765,7 +2771,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
@@ -2776,13 +2782,13 @@
         <v>4</v>
       </c>
       <c r="C12" t="s">
+        <v>185</v>
+      </c>
+      <c r="D12" t="s">
         <v>186</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>187</v>
-      </c>
-      <c r="E12" t="s">
-        <v>188</v>
       </c>
       <c r="F12" t="s">
         <v>152</v>
@@ -2803,7 +2809,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -2814,13 +2820,13 @@
         <v>5</v>
       </c>
       <c r="C13" t="s">
+        <v>189</v>
+      </c>
+      <c r="D13" t="s">
         <v>190</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>191</v>
-      </c>
-      <c r="E13" t="s">
-        <v>192</v>
       </c>
       <c r="F13" t="s">
         <v>152</v>
@@ -2841,7 +2847,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -2877,16 +2883,16 @@
         <v>7</v>
       </c>
       <c r="H1" t="s">
+        <v>202</v>
+      </c>
+      <c r="I1" t="s">
         <v>203</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>204</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>205</v>
-      </c>
-      <c r="K1" t="s">
-        <v>206</v>
       </c>
       <c r="L1" t="s">
         <v>11</v>
@@ -2900,19 +2906,19 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D2" t="s">
         <v>207</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>208</v>
-      </c>
-      <c r="E2" t="s">
-        <v>209</v>
       </c>
       <c r="F2" t="s">
         <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H2">
         <v>-320</v>
@@ -2924,10 +2930,10 @@
         <v>0</v>
       </c>
       <c r="K2" t="s">
+        <v>210</v>
+      </c>
+      <c r="L2" t="s">
         <v>211</v>
-      </c>
-      <c r="L2" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -2938,19 +2944,19 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D3" t="s">
         <v>213</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>214</v>
-      </c>
-      <c r="E3" t="s">
-        <v>215</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H3">
         <v>-320</v>
@@ -2962,10 +2968,10 @@
         <v>0</v>
       </c>
       <c r="K3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -2976,19 +2982,19 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
+        <v>216</v>
+      </c>
+      <c r="D4" t="s">
         <v>217</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>218</v>
-      </c>
-      <c r="E4" t="s">
-        <v>219</v>
       </c>
       <c r="F4" t="s">
         <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H4">
         <v>-320</v>
@@ -3000,10 +3006,10 @@
         <v>0</v>
       </c>
       <c r="K4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -3014,19 +3020,19 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
+        <v>220</v>
+      </c>
+      <c r="D5" t="s">
         <v>221</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>222</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>223</v>
       </c>
-      <c r="F5" t="s">
-        <v>224</v>
-      </c>
       <c r="G5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H5">
         <v>-100</v>
@@ -3038,10 +3044,10 @@
         <v>0</v>
       </c>
       <c r="K5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -3052,28 +3058,28 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D6" t="s">
+        <v>225</v>
+      </c>
+      <c r="E6" t="s">
         <v>226</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G6" t="s">
         <v>227</v>
       </c>
-      <c r="F6" t="s">
-        <v>224</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6" t="s">
+        <v>210</v>
+      </c>
+      <c r="L6" t="s">
         <v>228</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6" t="s">
-        <v>211</v>
-      </c>
-      <c r="L6" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -3084,28 +3090,28 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D7" t="s">
+        <v>229</v>
+      </c>
+      <c r="E7" t="s">
         <v>230</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
+        <v>223</v>
+      </c>
+      <c r="G7" t="s">
+        <v>227</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7" t="s">
+        <v>210</v>
+      </c>
+      <c r="L7" t="s">
         <v>231</v>
-      </c>
-      <c r="F7" t="s">
-        <v>224</v>
-      </c>
-      <c r="G7" t="s">
-        <v>228</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7" t="s">
-        <v>211</v>
-      </c>
-      <c r="L7" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
@@ -3116,28 +3122,28 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D8" t="s">
+        <v>232</v>
+      </c>
+      <c r="E8" t="s">
         <v>233</v>
-      </c>
-      <c r="E8" t="s">
-        <v>234</v>
       </c>
       <c r="F8" t="s">
         <v>17</v>
       </c>
       <c r="G8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
@@ -3148,28 +3154,28 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D9" t="s">
+        <v>235</v>
+      </c>
+      <c r="E9" t="s">
         <v>236</v>
-      </c>
-      <c r="E9" t="s">
-        <v>237</v>
       </c>
       <c r="F9" t="s">
         <v>17</v>
       </c>
       <c r="G9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
@@ -3180,28 +3186,28 @@
         <v>4</v>
       </c>
       <c r="C10" t="s">
+        <v>238</v>
+      </c>
+      <c r="D10" t="s">
         <v>239</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>240</v>
-      </c>
-      <c r="E10" t="s">
-        <v>241</v>
       </c>
       <c r="F10" t="s">
         <v>17</v>
       </c>
       <c r="G10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -3212,28 +3218,28 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
+        <v>242</v>
+      </c>
+      <c r="D11" t="s">
         <v>243</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>244</v>
-      </c>
-      <c r="E11" t="s">
-        <v>245</v>
       </c>
       <c r="F11" t="s">
         <v>147</v>
       </c>
       <c r="G11" t="s">
+        <v>209</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11" t="s">
         <v>210</v>
       </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11" t="s">
-        <v>211</v>
-      </c>
       <c r="L11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -3263,13 +3269,13 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>246</v>
+      </c>
+      <c r="G1" t="s">
         <v>247</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>248</v>
-      </c>
-      <c r="H1" t="s">
-        <v>249</v>
       </c>
       <c r="I1" t="s">
         <v>11</v>
@@ -3283,19 +3289,19 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
+        <v>249</v>
+      </c>
+      <c r="D2" t="s">
         <v>250</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>251</v>
-      </c>
-      <c r="E2" t="s">
-        <v>252</v>
       </c>
       <c r="F2" t="s">
         <v>17</v>
       </c>
       <c r="I2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -3306,19 +3312,19 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
+        <v>253</v>
+      </c>
+      <c r="D3" t="s">
         <v>254</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>255</v>
-      </c>
-      <c r="E3" t="s">
-        <v>256</v>
       </c>
       <c r="F3" t="s">
         <v>44</v>
       </c>
       <c r="I3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -3329,22 +3335,22 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
+        <v>257</v>
+      </c>
+      <c r="D4" t="s">
         <v>258</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>259</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>260</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>261</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>262</v>
-      </c>
-      <c r="I4" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -3355,22 +3361,22 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
+        <v>263</v>
+      </c>
+      <c r="D5" t="s">
         <v>264</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>265</v>
-      </c>
-      <c r="E5" t="s">
-        <v>266</v>
       </c>
       <c r="F5" t="s">
         <v>17</v>
       </c>
       <c r="H5" t="s">
+        <v>266</v>
+      </c>
+      <c r="I5" t="s">
         <v>267</v>
-      </c>
-      <c r="I5" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -3381,22 +3387,22 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
+        <v>268</v>
+      </c>
+      <c r="D6" t="s">
         <v>269</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>270</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>260</v>
+      </c>
+      <c r="G6" t="s">
+        <v>261</v>
+      </c>
+      <c r="I6" t="s">
         <v>271</v>
-      </c>
-      <c r="F6" t="s">
-        <v>261</v>
-      </c>
-      <c r="G6" t="s">
-        <v>262</v>
-      </c>
-      <c r="I6" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -3407,19 +3413,19 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
+        <v>272</v>
+      </c>
+      <c r="D7" t="s">
         <v>273</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>274</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
+        <v>260</v>
+      </c>
+      <c r="I7" t="s">
         <v>275</v>
-      </c>
-      <c r="F7" t="s">
-        <v>261</v>
-      </c>
-      <c r="I7" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -3430,22 +3436,22 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
+        <v>276</v>
+      </c>
+      <c r="D8" t="s">
         <v>277</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>278</v>
-      </c>
-      <c r="E8" t="s">
-        <v>279</v>
       </c>
       <c r="F8" t="s">
         <v>44</v>
       </c>
       <c r="H8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -3456,19 +3462,19 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
+        <v>280</v>
+      </c>
+      <c r="D9" t="s">
         <v>281</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>282</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>283</v>
       </c>
-      <c r="F9" t="s">
+      <c r="I9" t="s">
         <v>284</v>
-      </c>
-      <c r="I9" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -3479,22 +3485,22 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
+        <v>285</v>
+      </c>
+      <c r="D10" t="s">
         <v>286</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>287</v>
-      </c>
-      <c r="E10" t="s">
-        <v>288</v>
       </c>
       <c r="F10" t="s">
         <v>44</v>
       </c>
       <c r="G10" t="s">
+        <v>288</v>
+      </c>
+      <c r="I10" t="s">
         <v>289</v>
-      </c>
-      <c r="I10" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -3505,22 +3511,22 @@
         <v>9</v>
       </c>
       <c r="C11" t="s">
+        <v>290</v>
+      </c>
+      <c r="D11" t="s">
         <v>291</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>292</v>
-      </c>
-      <c r="E11" t="s">
-        <v>293</v>
       </c>
       <c r="F11" t="s">
         <v>17</v>
       </c>
       <c r="G11" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="I11" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -3531,19 +3537,19 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
+        <v>294</v>
+      </c>
+      <c r="D12" t="s">
         <v>295</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>296</v>
-      </c>
-      <c r="E12" t="s">
-        <v>297</v>
       </c>
       <c r="F12" t="s">
         <v>44</v>
       </c>
       <c r="I12" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -3554,19 +3560,19 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
+        <v>298</v>
+      </c>
+      <c r="D13" t="s">
         <v>299</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>300</v>
-      </c>
-      <c r="E13" t="s">
-        <v>301</v>
       </c>
       <c r="F13" t="s">
         <v>17</v>
       </c>
       <c r="I13" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance pressure sensor configurations and UI for Bang-Bang control
- Introduced a new function to parse trailing integers from labels for improved channel ID handling.
- Updated channel configurations to prefer explicit IDs for better alignment with UI and spreadsheet mappings.
- Enhanced the UI to visually tag Bang-Bang owned channels and display relevant device messages.
- Adjusted pressure sensor ranges and updated associated configurations to reflect new hardware specifications.
</commit_message>
<xml_diff>
--- a/sensor_config.xlsx
+++ b/sensor_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\GitHub\ERPL_GC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C0CC751-7630-4237-A0D2-199D27399BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DD38E71-B267-453A-B5F7-F42CF1ADF295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PT_Sensors" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,25 @@
     <sheet name="TC_Thermocouples" sheetId="3" r:id="rId3"/>
     <sheet name="DC_Solenoids" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="248">
   <si>
     <t>system</t>
   </si>
@@ -67,9 +80,6 @@
     <t>PT1E</t>
   </si>
   <si>
-    <t>PT1 LOX Reg Upstream</t>
-  </si>
-  <si>
     <t>pt1_lox_reg_up</t>
   </si>
   <si>
@@ -88,15 +98,6 @@
     <t>PT2E</t>
   </si>
   <si>
-    <t>PT2 LOX Reg Downstream</t>
-  </si>
-  <si>
-    <t>pt2_lox_reg_dn</t>
-  </si>
-  <si>
-    <t>1A043JCJI2E</t>
-  </si>
-  <si>
     <t>Downstream of LOX regulator</t>
   </si>
   <si>
@@ -148,9 +149,6 @@
     <t>PT11E</t>
   </si>
   <si>
-    <t>PT11 Fuel Reg Upstream</t>
-  </si>
-  <si>
     <t>pt11_fuel_reg_up</t>
   </si>
   <si>
@@ -166,18 +164,6 @@
     <t>PT12E</t>
   </si>
   <si>
-    <t>PT12 Fuel Reg Downstream</t>
-  </si>
-  <si>
-    <t>pt12_fuel_reg_dn</t>
-  </si>
-  <si>
-    <t>1A043JCGZIT</t>
-  </si>
-  <si>
-    <t>Fuel regulator downstream</t>
-  </si>
-  <si>
     <t>PT13E</t>
   </si>
   <si>
@@ -190,9 +176,6 @@
     <t>1A01WPHB22R</t>
   </si>
   <si>
-    <t>Fuel tank upstream</t>
-  </si>
-  <si>
     <t>PT14E</t>
   </si>
   <si>
@@ -322,198 +305,57 @@
     <t>PT1</t>
   </si>
   <si>
-    <t>BangBang Test</t>
-  </si>
-  <si>
-    <t>bb</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>Bang-bang controller test PT</t>
-  </si>
-  <si>
     <t>PT2</t>
   </si>
   <si>
-    <t>LOX Injector Pressure</t>
-  </si>
-  <si>
-    <t>pi_lox</t>
-  </si>
-  <si>
-    <t>LOX injector pressure</t>
-  </si>
-  <si>
     <t>PT3</t>
   </si>
   <si>
-    <t>Fuel Injector Pressure</t>
-  </si>
-  <si>
-    <t>pi_fuel</t>
-  </si>
-  <si>
-    <t>Fuel injector pressure</t>
-  </si>
-  <si>
     <t>PT4</t>
   </si>
   <si>
-    <t>LOX Tank Pressure</t>
-  </si>
-  <si>
-    <t>pt_lox</t>
-  </si>
-  <si>
-    <t>LOX tank pressure</t>
-  </si>
-  <si>
     <t>PT5</t>
   </si>
   <si>
-    <t>Fuel Tank Pressure</t>
-  </si>
-  <si>
-    <t>pt_fuel</t>
-  </si>
-  <si>
-    <t>Fuel tank pressure</t>
-  </si>
-  <si>
     <t>PT6</t>
   </si>
   <si>
-    <t>Pneumatic Supply</t>
-  </si>
-  <si>
-    <t>pt_pneu</t>
-  </si>
-  <si>
-    <t>pneumatic</t>
-  </si>
-  <si>
-    <t>Pneumatic supply pressure</t>
-  </si>
-  <si>
     <t>PT7</t>
   </si>
   <si>
-    <t>LOX Feed Pressure</t>
-  </si>
-  <si>
-    <t>pf_lox</t>
-  </si>
-  <si>
-    <t>LOX feed line pressure</t>
-  </si>
-  <si>
     <t>PT8</t>
   </si>
   <si>
-    <t>Fuel Feed Pressure</t>
-  </si>
-  <si>
-    <t>pf_fuel</t>
-  </si>
-  <si>
-    <t>Fuel feed line pressure</t>
-  </si>
-  <si>
     <t>PT9</t>
   </si>
   <si>
-    <t>LOX Vent Pressure</t>
-  </si>
-  <si>
-    <t>pv_lox</t>
-  </si>
-  <si>
-    <t>LOX vent pressure</t>
-  </si>
-  <si>
     <t>PT10</t>
   </si>
   <si>
-    <t>Fuel Vent Pressure</t>
-  </si>
-  <si>
-    <t>pv_fuel</t>
-  </si>
-  <si>
-    <t>Fuel vent pressure</t>
-  </si>
-  <si>
     <t>PT11</t>
   </si>
   <si>
-    <t>Purge Pressure</t>
-  </si>
-  <si>
-    <t>p_purge</t>
-  </si>
-  <si>
-    <t>Purge system pressure</t>
-  </si>
-  <si>
     <t>PT12</t>
   </si>
   <si>
-    <t>Ambient Pressure</t>
-  </si>
-  <si>
-    <t>p_amb</t>
-  </si>
-  <si>
     <t>ambient</t>
   </si>
   <si>
-    <t>Ambient/atmospheric reference</t>
-  </si>
-  <si>
     <t>PT13</t>
   </si>
   <si>
-    <t>PT Spare 13</t>
-  </si>
-  <si>
-    <t>pt13</t>
-  </si>
-  <si>
     <t>spare</t>
   </si>
   <si>
-    <t>Spare PT channel</t>
-  </si>
-  <si>
     <t>PT14</t>
   </si>
   <si>
-    <t>PT Spare 14</t>
-  </si>
-  <si>
-    <t>pt14</t>
-  </si>
-  <si>
     <t>PT15</t>
   </si>
   <si>
-    <t>PT Spare 15</t>
-  </si>
-  <si>
-    <t>pt15</t>
-  </si>
-  <si>
     <t>PT16</t>
   </si>
   <si>
-    <t>PT Spare 16</t>
-  </si>
-  <si>
-    <t>pt16</t>
-  </si>
-  <si>
     <t>cal_slope_a</t>
   </si>
   <si>
@@ -775,51 +617,18 @@
     <t>DC1</t>
   </si>
   <si>
-    <t>PB3 LOX Vent</t>
-  </si>
-  <si>
-    <t>pb3</t>
-  </si>
-  <si>
-    <t>LOX tank vent valve</t>
-  </si>
-  <si>
     <t>DC2</t>
   </si>
   <si>
-    <t>PB10 LOX Dump</t>
-  </si>
-  <si>
-    <t>pb10</t>
-  </si>
-  <si>
-    <t>LOX dump valve</t>
-  </si>
-  <si>
     <t>DC3</t>
   </si>
   <si>
-    <t>S2 Fuel Purge</t>
-  </si>
-  <si>
     <t>s2</t>
   </si>
   <si>
-    <t>misc</t>
-  </si>
-  <si>
-    <t>gn2_purge</t>
-  </si>
-  <si>
-    <t>Fuel side GN2 purge</t>
-  </si>
-  <si>
     <t>DC4</t>
   </si>
   <si>
-    <t>PB9 GOX Purge</t>
-  </si>
-  <si>
     <t>pb9</t>
   </si>
   <si>
@@ -832,105 +641,48 @@
     <t>DC5</t>
   </si>
   <si>
-    <t>S1 LOX Purge</t>
-  </si>
-  <si>
     <t>s1</t>
   </si>
   <si>
-    <t>LOX side GN2 purge</t>
-  </si>
-  <si>
     <t>DC6</t>
   </si>
   <si>
-    <t>S3 Muscle Purge</t>
-  </si>
-  <si>
     <t>s3</t>
   </si>
   <si>
-    <t>Pneumatic muscle purge</t>
-  </si>
-  <si>
     <t>DC7</t>
   </si>
   <si>
-    <t>PB7 Fuel Vent</t>
-  </si>
-  <si>
     <t>pb7</t>
   </si>
   <si>
-    <t>Fuel vent - bang-bang enabled</t>
-  </si>
-  <si>
     <t>DC8</t>
   </si>
   <si>
-    <t>PB1-5 Main Press Valves</t>
-  </si>
-  <si>
     <t>pb1-5</t>
   </si>
   <si>
-    <t>lox-fuel</t>
-  </si>
-  <si>
-    <t>Main pressurization valves</t>
-  </si>
-  <si>
     <t>DC9</t>
   </si>
   <si>
-    <t>PB8 Fuel Main Run</t>
-  </si>
-  <si>
     <t>pb8</t>
   </si>
   <si>
-    <t>run_valve</t>
-  </si>
-  <si>
-    <t>Fuel main run valve</t>
-  </si>
-  <si>
     <t>DC10</t>
   </si>
   <si>
-    <t>PB4 LOX Main Run</t>
-  </si>
-  <si>
     <t>pb4</t>
   </si>
   <si>
-    <t>LOX main run valve</t>
-  </si>
-  <si>
     <t>DC11</t>
   </si>
   <si>
-    <t>S6 Fuel Slow Press</t>
-  </si>
-  <si>
     <t>s6</t>
   </si>
   <si>
-    <t>Fuel slow pressurization</t>
-  </si>
-  <si>
     <t>DC12</t>
   </si>
   <si>
-    <t>S5 LOX Slow Press</t>
-  </si>
-  <si>
-    <t>s5</t>
-  </si>
-  <si>
-    <t>LOX slow pressurization</t>
-  </si>
-  <si>
     <t>TLCC</t>
   </si>
   <si>
@@ -938,6 +690,96 @@
   </si>
   <si>
     <t>Thrust load cell C</t>
+  </si>
+  <si>
+    <t>S2 fuel</t>
+  </si>
+  <si>
+    <t>Lox bb solenoid</t>
+  </si>
+  <si>
+    <t>fuel bb solenoid</t>
+  </si>
+  <si>
+    <t>S1 Lox</t>
+  </si>
+  <si>
+    <t>PB1 Lox</t>
+  </si>
+  <si>
+    <t>PB3 Lox</t>
+  </si>
+  <si>
+    <t>PB2</t>
+  </si>
+  <si>
+    <t>PB4 fuel</t>
+  </si>
+  <si>
+    <t>S4</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>runline</t>
+  </si>
+  <si>
+    <t>PB5</t>
+  </si>
+  <si>
+    <t>PB6</t>
+  </si>
+  <si>
+    <t>lox purge</t>
+  </si>
+  <si>
+    <t>fuel purge</t>
+  </si>
+  <si>
+    <t>muscle vent</t>
+  </si>
+  <si>
+    <t>Lox load</t>
+  </si>
+  <si>
+    <t>lox gn2 vent</t>
+  </si>
+  <si>
+    <t>fuel gn2 vent</t>
+  </si>
+  <si>
+    <t>lox runline</t>
+  </si>
+  <si>
+    <t>fuel runline</t>
+  </si>
+  <si>
+    <t>bb_lox</t>
+  </si>
+  <si>
+    <t>Fuel BangBang</t>
+  </si>
+  <si>
+    <t>bb_fuel</t>
+  </si>
+  <si>
+    <t>LOX  BangBang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lox Bang Bang </t>
+  </si>
+  <si>
+    <t>Fuel Bang Bang</t>
+  </si>
+  <si>
+    <t>PT1 LOX Sol Upstream</t>
+  </si>
+  <si>
+    <t>PT11 Fuel Sol Upstream</t>
+  </si>
+  <si>
+    <t>S4-5 fuel</t>
   </si>
 </sst>
 </file>
@@ -1278,9 +1120,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="10" max="10" width="17.88671875" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
+    <col min="10" max="10" width="17.77734375" customWidth="1"/>
     <col min="11" max="11" width="21.77734375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1332,33 +1175,6 @@
       <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
-      </c>
-      <c r="J2">
-        <v>10000</v>
-      </c>
-      <c r="K2">
-        <v>10000</v>
-      </c>
-      <c r="L2" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -1368,34 +1184,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3">
-        <v>4</v>
-      </c>
-      <c r="J3">
-        <v>1500</v>
-      </c>
-      <c r="K3">
-        <v>1500</v>
-      </c>
-      <c r="L3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -1406,34 +1195,34 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>245</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="G4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" t="s">
         <v>17</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
       </c>
       <c r="I4">
         <v>4</v>
       </c>
       <c r="J4">
-        <v>1500</v>
+        <v>10000</v>
       </c>
       <c r="K4">
-        <v>1500</v>
+        <v>10000</v>
       </c>
       <c r="L4" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -1444,22 +1233,22 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="G5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" t="s">
         <v>17</v>
-      </c>
-      <c r="H5" t="s">
-        <v>18</v>
       </c>
       <c r="I5">
         <v>4</v>
@@ -1471,7 +1260,7 @@
         <v>1500</v>
       </c>
       <c r="L5" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -1482,22 +1271,22 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" t="s">
         <v>17</v>
-      </c>
-      <c r="H6" t="s">
-        <v>18</v>
       </c>
       <c r="I6">
         <v>4</v>
@@ -1509,7 +1298,7 @@
         <v>1500</v>
       </c>
       <c r="L6" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -1520,34 +1309,34 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="H7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I7">
         <v>4</v>
       </c>
       <c r="J7">
-        <v>10000</v>
+        <v>1500</v>
       </c>
       <c r="K7">
-        <v>10000</v>
+        <v>1500</v>
       </c>
       <c r="L7" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
@@ -1558,34 +1347,34 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>246</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="H8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I8">
         <v>4</v>
       </c>
       <c r="J8">
-        <v>1500</v>
+        <v>10000</v>
       </c>
       <c r="K8">
-        <v>1500</v>
+        <v>10000</v>
       </c>
       <c r="L8" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
@@ -1596,34 +1385,34 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="F9" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="H9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I9">
         <v>4</v>
       </c>
       <c r="J9">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="K9">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="L9" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
@@ -1634,22 +1423,22 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="D10" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="G10" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="H10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I10">
         <v>4</v>
@@ -1661,7 +1450,7 @@
         <v>1500</v>
       </c>
       <c r="L10" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -1672,22 +1461,22 @@
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="D11" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="F11" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="G11" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="H11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I11">
         <v>4</v>
@@ -1699,7 +1488,7 @@
         <v>1500</v>
       </c>
       <c r="L11" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
@@ -1710,22 +1499,22 @@
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="D12" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="F12" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="G12" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I12">
         <v>4</v>
@@ -1737,7 +1526,7 @@
         <v>500</v>
       </c>
       <c r="L12" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -1748,22 +1537,22 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="D13" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="E13" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="F13" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="G13" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I13">
         <v>4</v>
@@ -1775,7 +1564,7 @@
         <v>2000</v>
       </c>
       <c r="L13" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
@@ -1786,22 +1575,22 @@
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="D14" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="E14" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="F14" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G14" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I14">
         <v>4</v>
@@ -1813,7 +1602,7 @@
         <v>1500</v>
       </c>
       <c r="L14" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
@@ -1824,22 +1613,22 @@
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="D15" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="G15" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I15">
         <v>4</v>
@@ -1851,7 +1640,7 @@
         <v>1500</v>
       </c>
       <c r="L15" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
@@ -1862,22 +1651,22 @@
         <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="D16" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="E16" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G16" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I16">
         <v>4</v>
@@ -1889,7 +1678,7 @@
         <v>1500</v>
       </c>
       <c r="L16" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
@@ -1900,22 +1689,22 @@
         <v>15</v>
       </c>
       <c r="C17" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="D17" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="E17" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="F17" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="G17" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I17">
         <v>4</v>
@@ -1927,423 +1716,225 @@
         <v>1500</v>
       </c>
       <c r="L17" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B18">
         <v>0</v>
       </c>
       <c r="C18" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="D18" t="s">
-        <v>99</v>
+        <v>242</v>
       </c>
       <c r="E18" t="s">
-        <v>100</v>
+        <v>239</v>
       </c>
       <c r="G18" t="s">
-        <v>101</v>
+        <v>16</v>
       </c>
       <c r="H18" t="s">
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="J18">
+        <v>1500</v>
+      </c>
+      <c r="K18">
+        <v>1500</v>
       </c>
       <c r="L18" t="s">
-        <v>102</v>
+        <v>243</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="D19" t="s">
-        <v>104</v>
+        <v>240</v>
       </c>
       <c r="E19" t="s">
-        <v>105</v>
+        <v>241</v>
       </c>
       <c r="G19" t="s">
+        <v>39</v>
+      </c>
+      <c r="H19" t="s">
         <v>17</v>
       </c>
-      <c r="H19" t="s">
-        <v>18</v>
+      <c r="J19">
+        <v>1500</v>
+      </c>
+      <c r="K19">
+        <v>1500</v>
       </c>
       <c r="L19" t="s">
-        <v>106</v>
+        <v>244</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B20">
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>107</v>
-      </c>
-      <c r="D20" t="s">
-        <v>108</v>
-      </c>
-      <c r="E20" t="s">
-        <v>109</v>
-      </c>
-      <c r="G20" t="s">
-        <v>44</v>
-      </c>
-      <c r="H20" t="s">
-        <v>18</v>
-      </c>
-      <c r="L20" t="s">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B21">
         <v>3</v>
       </c>
       <c r="C21" t="s">
-        <v>111</v>
-      </c>
-      <c r="D21" t="s">
-        <v>112</v>
-      </c>
-      <c r="E21" t="s">
-        <v>113</v>
-      </c>
-      <c r="G21" t="s">
-        <v>17</v>
-      </c>
-      <c r="H21" t="s">
-        <v>18</v>
-      </c>
-      <c r="L21" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B22">
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>115</v>
-      </c>
-      <c r="D22" t="s">
-        <v>116</v>
-      </c>
-      <c r="E22" t="s">
-        <v>117</v>
-      </c>
-      <c r="G22" t="s">
-        <v>44</v>
-      </c>
-      <c r="H22" t="s">
-        <v>18</v>
-      </c>
-      <c r="L22" t="s">
-        <v>118</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B23">
         <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D23" t="s">
-        <v>120</v>
-      </c>
-      <c r="E23" t="s">
-        <v>121</v>
-      </c>
-      <c r="G23" t="s">
-        <v>122</v>
-      </c>
-      <c r="H23" t="s">
-        <v>18</v>
-      </c>
-      <c r="L23" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B24">
         <v>6</v>
       </c>
       <c r="C24" t="s">
-        <v>124</v>
-      </c>
-      <c r="D24" t="s">
-        <v>125</v>
-      </c>
-      <c r="E24" t="s">
-        <v>126</v>
-      </c>
-      <c r="G24" t="s">
-        <v>17</v>
-      </c>
-      <c r="H24" t="s">
-        <v>18</v>
-      </c>
-      <c r="L24" t="s">
-        <v>127</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B25">
         <v>7</v>
       </c>
       <c r="C25" t="s">
-        <v>128</v>
-      </c>
-      <c r="D25" t="s">
-        <v>129</v>
-      </c>
-      <c r="E25" t="s">
-        <v>130</v>
-      </c>
-      <c r="G25" t="s">
-        <v>44</v>
-      </c>
-      <c r="H25" t="s">
-        <v>18</v>
-      </c>
-      <c r="L25" t="s">
-        <v>131</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B26">
         <v>8</v>
       </c>
       <c r="C26" t="s">
-        <v>132</v>
-      </c>
-      <c r="D26" t="s">
-        <v>133</v>
-      </c>
-      <c r="E26" t="s">
-        <v>134</v>
-      </c>
-      <c r="G26" t="s">
-        <v>17</v>
-      </c>
-      <c r="H26" t="s">
-        <v>18</v>
-      </c>
-      <c r="L26" t="s">
-        <v>135</v>
+        <v>96</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B27">
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>136</v>
-      </c>
-      <c r="D27" t="s">
-        <v>137</v>
-      </c>
-      <c r="E27" t="s">
-        <v>138</v>
-      </c>
-      <c r="G27" t="s">
-        <v>44</v>
-      </c>
-      <c r="H27" t="s">
-        <v>18</v>
-      </c>
-      <c r="L27" t="s">
-        <v>139</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B28">
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>140</v>
-      </c>
-      <c r="D28" t="s">
-        <v>141</v>
-      </c>
-      <c r="E28" t="s">
-        <v>142</v>
-      </c>
-      <c r="G28" t="s">
-        <v>122</v>
-      </c>
-      <c r="H28" t="s">
-        <v>18</v>
-      </c>
-      <c r="L28" t="s">
-        <v>143</v>
+        <v>98</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B29">
         <v>11</v>
       </c>
       <c r="C29" t="s">
-        <v>144</v>
-      </c>
-      <c r="D29" t="s">
-        <v>145</v>
-      </c>
-      <c r="E29" t="s">
-        <v>146</v>
-      </c>
-      <c r="G29" t="s">
-        <v>147</v>
-      </c>
-      <c r="H29" t="s">
-        <v>18</v>
-      </c>
-      <c r="L29" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B30">
         <v>12</v>
       </c>
       <c r="C30" t="s">
-        <v>149</v>
-      </c>
-      <c r="D30" t="s">
-        <v>150</v>
-      </c>
-      <c r="E30" t="s">
-        <v>151</v>
-      </c>
-      <c r="G30" t="s">
-        <v>152</v>
-      </c>
-      <c r="H30" t="s">
-        <v>18</v>
-      </c>
-      <c r="L30" t="s">
-        <v>153</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B31">
         <v>13</v>
       </c>
       <c r="C31" t="s">
-        <v>154</v>
-      </c>
-      <c r="D31" t="s">
-        <v>155</v>
-      </c>
-      <c r="E31" t="s">
-        <v>156</v>
-      </c>
-      <c r="G31" t="s">
-        <v>152</v>
-      </c>
-      <c r="H31" t="s">
-        <v>18</v>
-      </c>
-      <c r="L31" t="s">
-        <v>153</v>
+        <v>103</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B32">
         <v>14</v>
       </c>
       <c r="C32" t="s">
-        <v>157</v>
-      </c>
-      <c r="D32" t="s">
-        <v>158</v>
-      </c>
-      <c r="E32" t="s">
-        <v>159</v>
-      </c>
-      <c r="G32" t="s">
-        <v>152</v>
-      </c>
-      <c r="H32" t="s">
-        <v>18</v>
-      </c>
-      <c r="L32" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B33">
         <v>15</v>
       </c>
       <c r="C33" t="s">
-        <v>160</v>
-      </c>
-      <c r="D33" t="s">
-        <v>161</v>
-      </c>
-      <c r="E33" t="s">
-        <v>162</v>
-      </c>
-      <c r="G33" t="s">
-        <v>152</v>
-      </c>
-      <c r="H33" t="s">
-        <v>18</v>
-      </c>
-      <c r="L33" t="s">
-        <v>153</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -2354,7 +1945,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -2379,16 +1970,16 @@
         <v>7</v>
       </c>
       <c r="H1" t="s">
-        <v>163</v>
+        <v>106</v>
       </c>
       <c r="I1" t="s">
-        <v>164</v>
+        <v>107</v>
       </c>
       <c r="J1" t="s">
-        <v>165</v>
+        <v>108</v>
       </c>
       <c r="K1" t="s">
-        <v>166</v>
+        <v>109</v>
       </c>
       <c r="L1" t="s">
         <v>11</v>
@@ -2402,19 +1993,19 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>167</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
-        <v>168</v>
+        <v>111</v>
       </c>
       <c r="E2" t="s">
-        <v>169</v>
+        <v>112</v>
       </c>
       <c r="F2" t="s">
-        <v>170</v>
+        <v>113</v>
       </c>
       <c r="G2" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H2">
         <v>296590</v>
@@ -2429,7 +2020,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>172</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -2440,19 +2031,19 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>173</v>
+        <v>116</v>
       </c>
       <c r="D3" t="s">
-        <v>174</v>
+        <v>117</v>
       </c>
       <c r="E3" t="s">
-        <v>175</v>
+        <v>118</v>
       </c>
       <c r="F3" t="s">
-        <v>170</v>
+        <v>113</v>
       </c>
       <c r="G3" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H3">
         <v>59447</v>
@@ -2467,7 +2058,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>176</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -2478,19 +2069,19 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>177</v>
+        <v>120</v>
       </c>
       <c r="D4" t="s">
-        <v>302</v>
+        <v>215</v>
       </c>
       <c r="E4" t="s">
-        <v>303</v>
+        <v>216</v>
       </c>
       <c r="F4" t="s">
-        <v>170</v>
+        <v>113</v>
       </c>
       <c r="G4" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H4">
         <v>59447.9</v>
@@ -2505,7 +2096,7 @@
         <v>130</v>
       </c>
       <c r="L4" t="s">
-        <v>304</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -2516,19 +2107,19 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>181</v>
+        <v>124</v>
       </c>
       <c r="D5" t="s">
-        <v>182</v>
+        <v>125</v>
       </c>
       <c r="E5" t="s">
-        <v>183</v>
+        <v>126</v>
       </c>
       <c r="F5" t="s">
-        <v>180</v>
+        <v>123</v>
       </c>
       <c r="G5" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H5">
         <v>59447</v>
@@ -2543,7 +2134,7 @@
         <v>129</v>
       </c>
       <c r="L5" t="s">
-        <v>184</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -2554,19 +2145,19 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>185</v>
+        <v>128</v>
       </c>
       <c r="D6" t="s">
-        <v>186</v>
+        <v>129</v>
       </c>
       <c r="E6" t="s">
-        <v>187</v>
+        <v>130</v>
       </c>
       <c r="F6" t="s">
-        <v>152</v>
+        <v>102</v>
       </c>
       <c r="G6" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H6">
         <v>1000000</v>
@@ -2581,7 +2172,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>188</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -2592,19 +2183,19 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>189</v>
+        <v>132</v>
       </c>
       <c r="D7" t="s">
-        <v>190</v>
+        <v>133</v>
       </c>
       <c r="E7" t="s">
-        <v>191</v>
+        <v>134</v>
       </c>
       <c r="F7" t="s">
-        <v>152</v>
+        <v>102</v>
       </c>
       <c r="G7" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H7">
         <v>1000000</v>
@@ -2619,30 +2210,30 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>192</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B8">
         <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>167</v>
+        <v>110</v>
       </c>
       <c r="D8" t="s">
-        <v>193</v>
+        <v>136</v>
       </c>
       <c r="E8" t="s">
-        <v>170</v>
+        <v>113</v>
       </c>
       <c r="F8" t="s">
-        <v>170</v>
+        <v>113</v>
       </c>
       <c r="G8" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H8">
         <v>1000000</v>
@@ -2657,30 +2248,30 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>194</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>173</v>
+        <v>116</v>
       </c>
       <c r="D9" t="s">
-        <v>182</v>
+        <v>125</v>
       </c>
       <c r="E9" t="s">
-        <v>183</v>
+        <v>126</v>
       </c>
       <c r="F9" t="s">
-        <v>180</v>
+        <v>123</v>
       </c>
       <c r="G9" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H9">
         <v>500000</v>
@@ -2695,30 +2286,30 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>195</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B10">
         <v>2</v>
       </c>
       <c r="C10" t="s">
-        <v>177</v>
+        <v>120</v>
       </c>
       <c r="D10" t="s">
-        <v>178</v>
+        <v>121</v>
       </c>
       <c r="E10" t="s">
-        <v>179</v>
+        <v>122</v>
       </c>
       <c r="F10" t="s">
-        <v>180</v>
+        <v>123</v>
       </c>
       <c r="G10" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H10">
         <v>300000</v>
@@ -2733,30 +2324,30 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>196</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B11">
         <v>3</v>
       </c>
       <c r="C11" t="s">
-        <v>181</v>
+        <v>124</v>
       </c>
       <c r="D11" t="s">
-        <v>197</v>
+        <v>140</v>
       </c>
       <c r="E11" t="s">
-        <v>198</v>
+        <v>141</v>
       </c>
       <c r="F11" t="s">
-        <v>199</v>
+        <v>142</v>
       </c>
       <c r="G11" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H11">
         <v>100000</v>
@@ -2771,30 +2362,30 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>200</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B12">
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>185</v>
+        <v>128</v>
       </c>
       <c r="D12" t="s">
-        <v>186</v>
+        <v>129</v>
       </c>
       <c r="E12" t="s">
-        <v>187</v>
+        <v>130</v>
       </c>
       <c r="F12" t="s">
-        <v>152</v>
+        <v>102</v>
       </c>
       <c r="G12" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H12">
         <v>1000000</v>
@@ -2809,30 +2400,30 @@
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>201</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B13">
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>189</v>
+        <v>132</v>
       </c>
       <c r="D13" t="s">
-        <v>190</v>
+        <v>133</v>
       </c>
       <c r="E13" t="s">
-        <v>191</v>
+        <v>134</v>
       </c>
       <c r="F13" t="s">
-        <v>152</v>
+        <v>102</v>
       </c>
       <c r="G13" t="s">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="H13">
         <v>1000000</v>
@@ -2847,7 +2438,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>201</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -2858,7 +2449,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -2883,16 +2474,16 @@
         <v>7</v>
       </c>
       <c r="H1" t="s">
-        <v>202</v>
+        <v>145</v>
       </c>
       <c r="I1" t="s">
-        <v>203</v>
+        <v>146</v>
       </c>
       <c r="J1" t="s">
-        <v>204</v>
+        <v>147</v>
       </c>
       <c r="K1" t="s">
-        <v>205</v>
+        <v>148</v>
       </c>
       <c r="L1" t="s">
         <v>11</v>
@@ -2906,19 +2497,19 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>206</v>
+        <v>149</v>
       </c>
       <c r="D2" t="s">
-        <v>207</v>
+        <v>150</v>
       </c>
       <c r="E2" t="s">
-        <v>208</v>
+        <v>151</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>209</v>
+        <v>152</v>
       </c>
       <c r="H2">
         <v>-320</v>
@@ -2930,10 +2521,10 @@
         <v>0</v>
       </c>
       <c r="K2" t="s">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="L2" t="s">
-        <v>211</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -2944,19 +2535,19 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>212</v>
+        <v>155</v>
       </c>
       <c r="D3" t="s">
-        <v>213</v>
+        <v>156</v>
       </c>
       <c r="E3" t="s">
-        <v>214</v>
+        <v>157</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>209</v>
+        <v>152</v>
       </c>
       <c r="H3">
         <v>-320</v>
@@ -2968,10 +2559,10 @@
         <v>0</v>
       </c>
       <c r="K3" t="s">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="L3" t="s">
-        <v>215</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -2982,19 +2573,19 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>216</v>
+        <v>159</v>
       </c>
       <c r="D4" t="s">
-        <v>217</v>
+        <v>160</v>
       </c>
       <c r="E4" t="s">
-        <v>218</v>
+        <v>161</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>209</v>
+        <v>152</v>
       </c>
       <c r="H4">
         <v>-320</v>
@@ -3006,10 +2597,10 @@
         <v>0</v>
       </c>
       <c r="K4" t="s">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="L4" t="s">
-        <v>219</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -3020,19 +2611,19 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>220</v>
+        <v>163</v>
       </c>
       <c r="D5" t="s">
-        <v>221</v>
+        <v>164</v>
       </c>
       <c r="E5" t="s">
-        <v>222</v>
+        <v>165</v>
       </c>
       <c r="F5" t="s">
-        <v>223</v>
+        <v>166</v>
       </c>
       <c r="G5" t="s">
-        <v>209</v>
+        <v>152</v>
       </c>
       <c r="H5">
         <v>-100</v>
@@ -3044,202 +2635,202 @@
         <v>0</v>
       </c>
       <c r="K5" t="s">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="L5" t="s">
-        <v>224</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B6">
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>206</v>
+        <v>149</v>
       </c>
       <c r="D6" t="s">
-        <v>225</v>
+        <v>168</v>
       </c>
       <c r="E6" t="s">
-        <v>226</v>
+        <v>169</v>
       </c>
       <c r="F6" t="s">
-        <v>223</v>
+        <v>166</v>
       </c>
       <c r="G6" t="s">
-        <v>227</v>
+        <v>170</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6" t="s">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="L6" t="s">
-        <v>228</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>212</v>
+        <v>155</v>
       </c>
       <c r="D7" t="s">
-        <v>229</v>
+        <v>172</v>
       </c>
       <c r="E7" t="s">
-        <v>230</v>
+        <v>173</v>
       </c>
       <c r="F7" t="s">
-        <v>223</v>
+        <v>166</v>
       </c>
       <c r="G7" t="s">
-        <v>227</v>
+        <v>170</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7" t="s">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="L7" t="s">
-        <v>231</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>216</v>
+        <v>159</v>
       </c>
       <c r="D8" t="s">
-        <v>232</v>
+        <v>175</v>
       </c>
       <c r="E8" t="s">
-        <v>233</v>
+        <v>176</v>
       </c>
       <c r="F8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G8" t="s">
-        <v>227</v>
+        <v>170</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8" t="s">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="L8" t="s">
-        <v>234</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B9">
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>220</v>
+        <v>163</v>
       </c>
       <c r="D9" t="s">
-        <v>235</v>
+        <v>178</v>
       </c>
       <c r="E9" t="s">
-        <v>236</v>
+        <v>179</v>
       </c>
       <c r="F9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G9" t="s">
-        <v>227</v>
+        <v>170</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9" t="s">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="L9" t="s">
-        <v>237</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B10">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>238</v>
+        <v>181</v>
       </c>
       <c r="D10" t="s">
-        <v>239</v>
+        <v>182</v>
       </c>
       <c r="E10" t="s">
-        <v>240</v>
+        <v>183</v>
       </c>
       <c r="F10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G10" t="s">
-        <v>227</v>
+        <v>170</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10" t="s">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="L10" t="s">
-        <v>241</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B11">
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>242</v>
+        <v>185</v>
       </c>
       <c r="D11" t="s">
-        <v>243</v>
+        <v>186</v>
       </c>
       <c r="E11" t="s">
-        <v>244</v>
+        <v>187</v>
       </c>
       <c r="F11" t="s">
-        <v>147</v>
+        <v>100</v>
       </c>
       <c r="G11" t="s">
-        <v>209</v>
+        <v>152</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11" t="s">
-        <v>210</v>
+        <v>153</v>
       </c>
       <c r="L11" t="s">
-        <v>245</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -3250,7 +2841,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -3269,13 +2860,13 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>246</v>
+        <v>189</v>
       </c>
       <c r="G1" t="s">
-        <v>247</v>
+        <v>190</v>
       </c>
       <c r="H1" t="s">
-        <v>248</v>
+        <v>191</v>
       </c>
       <c r="I1" t="s">
         <v>11</v>
@@ -3283,296 +2874,278 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>249</v>
+        <v>192</v>
       </c>
       <c r="D2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E2" t="s">
-        <v>251</v>
+        <v>221</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>252</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>253</v>
+        <v>193</v>
       </c>
       <c r="D3" t="s">
-        <v>254</v>
-      </c>
-      <c r="E3" t="s">
-        <v>255</v>
+        <v>218</v>
       </c>
       <c r="F3" t="s">
-        <v>44</v>
+        <v>39</v>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>256</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>257</v>
+        <v>194</v>
       </c>
       <c r="D4" t="s">
-        <v>258</v>
+        <v>222</v>
       </c>
       <c r="E4" t="s">
-        <v>259</v>
+        <v>195</v>
       </c>
       <c r="F4" t="s">
-        <v>260</v>
-      </c>
-      <c r="G4" t="s">
-        <v>261</v>
+        <v>16</v>
       </c>
       <c r="I4" t="s">
-        <v>262</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B5">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>263</v>
+        <v>196</v>
       </c>
       <c r="D5" t="s">
-        <v>264</v>
+        <v>223</v>
       </c>
       <c r="E5" t="s">
-        <v>265</v>
+        <v>197</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H5" t="s">
-        <v>266</v>
+        <v>198</v>
       </c>
       <c r="I5" t="s">
-        <v>267</v>
+        <v>236</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B6">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>268</v>
+        <v>204</v>
       </c>
       <c r="D6" t="s">
-        <v>269</v>
+        <v>226</v>
       </c>
       <c r="E6" t="s">
-        <v>270</v>
+        <v>205</v>
       </c>
       <c r="F6" t="s">
-        <v>260</v>
-      </c>
-      <c r="G6" t="s">
-        <v>261</v>
+        <v>16</v>
+      </c>
+      <c r="H6" t="s">
+        <v>198</v>
       </c>
       <c r="I6" t="s">
-        <v>271</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B7">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>272</v>
+        <v>208</v>
       </c>
       <c r="D7" t="s">
-        <v>273</v>
+        <v>227</v>
       </c>
       <c r="E7" t="s">
-        <v>274</v>
+        <v>209</v>
       </c>
       <c r="F7" t="s">
-        <v>260</v>
+        <v>39</v>
       </c>
       <c r="I7" t="s">
-        <v>275</v>
+        <v>233</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B8">
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>276</v>
+        <v>200</v>
       </c>
       <c r="D8" t="s">
-        <v>277</v>
+        <v>224</v>
       </c>
       <c r="E8" t="s">
-        <v>278</v>
+        <v>201</v>
       </c>
       <c r="F8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" t="s">
-        <v>266</v>
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
+        <v>228</v>
       </c>
       <c r="I8" t="s">
-        <v>279</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B9">
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>280</v>
+        <v>202</v>
       </c>
       <c r="D9" t="s">
-        <v>281</v>
+        <v>225</v>
       </c>
       <c r="E9" t="s">
-        <v>282</v>
+        <v>203</v>
       </c>
       <c r="F9" t="s">
-        <v>283</v>
+        <v>39</v>
+      </c>
+      <c r="G9" t="s">
+        <v>228</v>
       </c>
       <c r="I9" t="s">
-        <v>284</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B10">
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>285</v>
+        <v>206</v>
       </c>
       <c r="D10" t="s">
-        <v>286</v>
+        <v>247</v>
       </c>
       <c r="E10" t="s">
-        <v>287</v>
+        <v>207</v>
       </c>
       <c r="F10" t="s">
-        <v>44</v>
-      </c>
-      <c r="G10" t="s">
-        <v>288</v>
+        <v>39</v>
       </c>
       <c r="I10" t="s">
-        <v>289</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B11">
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>290</v>
+        <v>210</v>
       </c>
       <c r="D11" t="s">
-        <v>291</v>
+        <v>229</v>
       </c>
       <c r="E11" t="s">
-        <v>292</v>
+        <v>211</v>
       </c>
       <c r="F11" t="s">
-        <v>17</v>
-      </c>
-      <c r="G11" t="s">
-        <v>288</v>
+        <v>16</v>
       </c>
       <c r="I11" t="s">
-        <v>293</v>
+        <v>234</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B12">
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>294</v>
+        <v>212</v>
       </c>
       <c r="D12" t="s">
-        <v>295</v>
+        <v>230</v>
       </c>
       <c r="E12" t="s">
-        <v>296</v>
+        <v>213</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="I12" t="s">
-        <v>297</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B13">
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>298</v>
-      </c>
-      <c r="D13" t="s">
-        <v>299</v>
-      </c>
-      <c r="E13" t="s">
-        <v>300</v>
-      </c>
-      <c r="F13" t="s">
-        <v>17</v>
-      </c>
-      <c r="I13" t="s">
-        <v>301</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>